<commit_message>
Fan link included in parts document
</commit_message>
<xml_diff>
--- a/Documents/Dev-Files/Raspi-ZUUL/Documents/Component-Selection.xlsx
+++ b/Documents/Dev-Files/Raspi-ZUUL/Documents/Component-Selection.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24704"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\AdamLucks-GateSecuritySystem\Documents\Dev-Files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\AdamLucks-GateSecuritySystem\Documents\Dev-Files\Raspi-ZUUL\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1493A5D0-B035-4A75-9565-F545DA870DDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E76CFBE-22D2-482D-8337-082EE2AED4E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="32">
   <si>
     <t>S.No</t>
   </si>
@@ -112,6 +112,15 @@
   </si>
   <si>
     <t>Will be ordered by Sir Hassan internationally. Link provided</t>
+  </si>
+  <si>
+    <t>Raspberry Pi 4 Fan</t>
+  </si>
+  <si>
+    <t>RASPBERRY PI 4 CASING FAN</t>
+  </si>
+  <si>
+    <t>Used to keep the Raspberry Pi cool under heavy processing applications</t>
   </si>
 </sst>
 </file>
@@ -154,7 +163,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -262,12 +271,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -312,6 +332,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -319,6 +340,26 @@
   </cellStyles>
   <dxfs count="12">
     <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -333,26 +374,6 @@
         </bottom>
         <vertical/>
         <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -559,7 +580,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{015DB811-CAAB-4CD9-A1D4-1C92075F62AD}" name="Table1" displayName="Table1" ref="A1:H6" totalsRowShown="0" headerRowDxfId="11" headerRowBorderDxfId="10" tableBorderDxfId="9" totalsRowBorderDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{015DB811-CAAB-4CD9-A1D4-1C92075F62AD}" name="Table1" displayName="Table1" ref="A1:H7" totalsRowShown="0" headerRowDxfId="11" headerRowBorderDxfId="10" tableBorderDxfId="9" totalsRowBorderDxfId="8">
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{18F54C0B-A7E8-4071-9EBF-DB3126C9CDE9}" name="S.No" dataDxfId="7"/>
     <tableColumn id="2" xr3:uid="{317E679B-3A79-40C4-9272-4E4E6E311408}" name="Component Name" dataDxfId="6"/>
@@ -567,8 +588,8 @@
     <tableColumn id="4" xr3:uid="{CF1C59C6-6EE5-49E0-9094-40F8CE5E87A8}" name="Quantity" dataDxfId="4"/>
     <tableColumn id="5" xr3:uid="{0DEF5A6D-DB44-4743-864E-972C7CD936F7}" name="Cost" dataDxfId="3"/>
     <tableColumn id="6" xr3:uid="{A04DEE05-1D8F-43F3-A2DF-1BF2819B85CD}" name="Reference Link" dataDxfId="2" dataCellStyle="Hyperlink"/>
-    <tableColumn id="8" xr3:uid="{564315F0-111A-448F-8B4B-0DEE1B8A0A94}" name="Local Link" dataDxfId="0" dataCellStyle="Hyperlink"/>
-    <tableColumn id="7" xr3:uid="{46EC11C6-2EAF-4885-9B5D-F5A79DA3565B}" name="Remarks" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{564315F0-111A-448F-8B4B-0DEE1B8A0A94}" name="Local Link" dataDxfId="1" dataCellStyle="Hyperlink"/>
+    <tableColumn id="7" xr3:uid="{46EC11C6-2EAF-4885-9B5D-F5A79DA3565B}" name="Remarks" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1006,10 +1027,30 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="D7" s="1"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
+      <c r="A7" s="20">
+        <v>6</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="10">
+        <v>1</v>
+      </c>
+      <c r="E7" s="11">
+        <v>5.0599999999999996</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="G7" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" s="13" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D8" s="1"/>
@@ -1153,11 +1194,12 @@
     <hyperlink ref="G2" r:id="rId6" xr:uid="{57C3F10E-C9EC-442F-B544-CC0FB66C187B}"/>
     <hyperlink ref="G3" r:id="rId7" xr:uid="{FDC73A8A-2B36-4377-953E-26FB7E348CED}"/>
     <hyperlink ref="G4" r:id="rId8" xr:uid="{6C39B9F5-6B06-4EFA-9DB2-FA4C3A86BBDD}"/>
+    <hyperlink ref="F7" r:id="rId9" xr:uid="{8B90FC5D-3B35-43B3-8E10-EAEAAF651675}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId9"/>
+  <pageSetup orientation="portrait" r:id="rId10"/>
   <tableParts count="1">
-    <tablePart r:id="rId10"/>
+    <tablePart r:id="rId11"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>